<commit_message>
refactor: optimize partner validation rules
</commit_message>
<xml_diff>
--- a/docs/validation_rules_inventory.xlsx
+++ b/docs/validation_rules_inventory.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Incohérences" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Règles'!$A$2:$W$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Règles'!$A$2:$W$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Incohérences'!$A$2:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -172,8 +172,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationRules" displayName="ValidationRules" ref="A2:W48" headerRowCount="1">
-  <autoFilter ref="A2:W48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationRules" displayName="ValidationRules" ref="A2:W44" headerRowCount="1">
+  <autoFilter ref="A2:W44"/>
   <tableColumns count="23">
     <tableColumn id="1" name="Code canonique"/>
     <tableColumn id="2" name="Alias / anciens codes"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W48"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -928,12 +928,12 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Mettre en revue</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -1549,7 +1549,11 @@
           <t>MASTERDATA_MISSING</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SOLDTO_MASTERDATA_UNAVAILABLE</t>
+        </is>
+      </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Masterdata Missing</t>
@@ -1646,7 +1650,11 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : SOLDTO_MASTERDATA_UNAVAILABLE</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2176,33 +2184,33 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>CONTRACT_BREAK_ADDRESSES_MISSING</t>
+          <t>CONTRACT_BREAK_ARTICLES_MISSING</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Contract Break Addresses Missing</t>
+          <t>Contract Break Articles Missing</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse exploitable n'a été trouvée pour résoudre le SHIP-TO.</t>
+          <t>Aucune ligne article exploitable n'a été trouvée.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>EXTRACTION</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -2247,17 +2255,17 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse exploitable n'a été trouvée pour résoudre le SHIP-TO.</t>
+          <t>Aucune ligne article exploitable n'a été trouvée.</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>No usable address was found to resolve the SHIP-TO.</t>
+          <t>No usable order line item was found.</t>
         </is>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr"/>
@@ -2281,33 +2289,37 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>CONTRACT_BREAK_ARTICLES_MISSING</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr"/>
+          <t>SOLDTO_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
+        </is>
+      </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Contract Break Articles Missing</t>
+          <t>Soldto Not Found</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article exploitable n'a été trouvée.</t>
+          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>EXTRACTION</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Référentiel / matching</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -2352,20 +2364,24 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article exploitable n'a été trouvée.</t>
+          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>No usable order line item was found.</t>
+          <t>No matching SOLD-TO was found in master data.</t>
         </is>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S18" s="4" t="inlineStr"/>
+          <t>app/engines/rejection_engine.py</t>
+        </is>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>_check_customer</t>
+        </is>
+      </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2378,26 +2394,30 @@
       </c>
       <c r="V18" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W18" s="4" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>CONTRACT_BREAK_SOLDTO_MISSING</t>
+          <t>SOLDTO_AMBIGUOUS_MATCH</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr"/>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Contract Break Soldto Missing</t>
+          <t>Soldto Ambiguous Match</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Le SOLD-TO n'a pas pu être déterminé.</t>
+          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2457,12 +2477,12 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>Le SOLD-TO n'a pas pu être déterminé.</t>
+          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>The SOLD-TO could not be resolved.</t>
+          <t>Multiple SOLD-TO candidates matched with equivalent confidence.</t>
         </is>
       </c>
       <c r="R19" s="4" t="inlineStr">
@@ -2491,18 +2511,22 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>SHIPTO_CANDIDATES_MISSING</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr"/>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Contract Break Shipto Candidates Missing</t>
+          <t>Shipto Candidates Missing</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Aucun candidat SHIP-TO n'a été trouvé dans la famille SOLD-TO.</t>
+          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2542,12 +2566,12 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -2562,12 +2586,12 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>Aucun candidat SHIP-TO n'a été trouvé dans la famille SOLD-TO.</t>
+          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>No SHIP-TO candidate was found in the SOLD-TO family.</t>
+          <t>No SHIP-TO candidate exists in the current SOLD-TO family.</t>
         </is>
       </c>
       <c r="R20" s="4" t="inlineStr">
@@ -2591,23 +2615,31 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SOLDTO_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr"/>
+          <t>SHIPTO_NO_STRONG_MATCH</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
+        </is>
+      </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Soldto Not Found</t>
+          <t>Shipto No Strong Match</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
+          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2667,12 +2699,12 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
+          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
         </is>
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>No matching SOLD-TO was found in master data.</t>
+          <t>SHIP-TO candidates exist but none matched with strong evidence.</t>
         </is>
       </c>
       <c r="R21" s="4" t="inlineStr">
@@ -2680,7 +2712,11 @@
           <t>app/engines/rejection_engine.py</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>_check_delivery_address</t>
+        </is>
+      </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2693,26 +2729,30 @@
       </c>
       <c r="V21" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W21" s="4" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="W21" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>SOLDTO_AMBIGUOUS_MATCH</t>
+          <t>SHIPTO_AMBIGUOUS_MATCH</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Soldto Ambiguous Match</t>
+          <t>Shipto Ambiguous Match</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
+          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2772,12 +2812,12 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
+          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>Multiple SOLD-TO candidates matched with equivalent confidence.</t>
+          <t>Multiple SHIP-TO candidates matched with equivalent strong evidence.</t>
         </is>
       </c>
       <c r="R22" s="4" t="inlineStr">
@@ -2806,18 +2846,18 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
+          <t>SHIPTO_SOLDTO_MISMATCH</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr"/>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Shipto Weak Evidence In Soldto Family</t>
+          <t>Shipto Soldto Mismatch</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO n'a pas de preuve forte code postal ou ville. Une rue seule est insuffisante.</t>
+          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -2857,12 +2897,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -2877,12 +2917,12 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO n'a pas de preuve forte code postal ou ville. Une rue seule est insuffisante.</t>
+          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>The SHIP-TO has no strong postal-code or city evidence. Street-only is not sufficient.</t>
+          <t>The selected SHIP-TO does not belong to the current SOLD-TO family.</t>
         </is>
       </c>
       <c r="R23" s="4" t="inlineStr">
@@ -2911,37 +2951,33 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_NO_STRONG_MATCH</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>SHIPTO_MISSING</t>
-        </is>
-      </c>
+          <t>EDIFACT_MISSING_BGM</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr"/>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Shipto No Strong Match</t>
+          <t>Edifact Missing Bgm</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
+          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>EDI_VALIDATION</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -2956,7 +2992,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -2966,7 +3002,7 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -2986,17 +3022,17 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
+          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>SHIP-TO candidates exist but none matched with strong evidence.</t>
+          <t>The EDIFACT BGM segment is missing the mandatory order reference.</t>
         </is>
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S24" s="4" t="inlineStr"/>
@@ -3015,42 +3051,38 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : SHIPTO_MISSING</t>
-        </is>
-      </c>
+      <c r="W24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_AMBIGUOUS_MATCH</t>
+          <t>EDIFACT_MISSING_DTM_137</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Shipto Ambiguous Match</t>
+          <t>Edifact Missing Dtm 137</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
+          <t>La date document DTM+137 est manquante ou invalide.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>EDI_VALIDATION</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -3065,7 +3097,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -3075,7 +3107,7 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -3095,17 +3127,17 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
+          <t>La date document DTM+137 est manquante ou invalide.</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>Multiple SHIP-TO candidates matched with equivalent strong evidence.</t>
+          <t>The DTM+137 document date is missing or invalid.</t>
         </is>
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S25" s="4" t="inlineStr"/>
@@ -3129,18 +3161,18 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_BGM</t>
+          <t>EDIFACT_MISSING_NAD_BY</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr"/>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Bgm</t>
+          <t>Edifact Missing Nad By</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
+          <t>Le segment acheteur NAD+BY est incomplet.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -3200,12 +3232,12 @@
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
+          <t>Le segment acheteur NAD+BY est incomplet.</t>
         </is>
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT BGM segment is missing the mandatory order reference.</t>
+          <t>The buyer NAD+BY segment is incomplete.</t>
         </is>
       </c>
       <c r="R26" s="4" t="inlineStr">
@@ -3234,18 +3266,18 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_DTM_137</t>
+          <t>EDIFACT_MISSING_NAD_DP</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Dtm 137</t>
+          <t>Edifact Missing Nad Dp</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>La date document DTM+137 est manquante ou invalide.</t>
+          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -3305,12 +3337,12 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>La date document DTM+137 est manquante ou invalide.</t>
+          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
         </is>
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>The DTM+137 document date is missing or invalid.</t>
+          <t>The delivery NAD+DP segment is incomplete or unresolved.</t>
         </is>
       </c>
       <c r="R27" s="4" t="inlineStr">
@@ -3339,18 +3371,18 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_NAD_BY</t>
+          <t>EDIFACT_MISSING_LIN</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr"/>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Nad By</t>
+          <t>Edifact Missing Lin</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Le segment acheteur NAD+BY est incomplet.</t>
+          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -3410,12 +3442,12 @@
       </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
-          <t>Le segment acheteur NAD+BY est incomplet.</t>
+          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
         </is>
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>The buyer NAD+BY segment is incomplete.</t>
+          <t>The EDIFACT line segments LIN/PIA/IMD/QTY/PRI are missing or incomplete.</t>
         </is>
       </c>
       <c r="R28" s="4" t="inlineStr">
@@ -3444,23 +3476,27 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_NAD_DP</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr"/>
+          <t>ARTICLE_QUANTITY_INVALID</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>INVALID_QUANTITY, QUANTITY_INVALID</t>
+        </is>
+      </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Nad Dp</t>
+          <t>Article Quantity Invalid</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
+          <t>Une ou plusieurs quantités article sont invalides.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3470,12 +3506,12 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -3485,7 +3521,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -3515,17 +3551,17 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
+          <t>Une ou plusieurs quantités article sont invalides.</t>
         </is>
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>The delivery NAD+DP segment is incomplete or unresolved.</t>
+          <t>One or more article quantities are invalid.</t>
         </is>
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S29" s="4" t="inlineStr"/>
@@ -3544,28 +3580,32 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : INVALID_QUANTITY, QUANTITY_INVALID</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_LIN</t>
+          <t>UNIT_PRICE_MISSING</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr"/>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Lin</t>
+          <t>Unit Price Missing</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
+          <t>Un ou plusieurs prix unitaires sont manquants.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3575,12 +3615,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -3590,7 +3630,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
@@ -3620,17 +3660,17 @@
       </c>
       <c r="P30" s="4" t="inlineStr">
         <is>
-          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
+          <t>Un ou plusieurs prix unitaires sont manquants.</t>
         </is>
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT line segments LIN/PIA/IMD/QTY/PRI are missing or incomplete.</t>
+          <t>One or more unit prices are missing.</t>
         </is>
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S30" s="4" t="inlineStr"/>
@@ -3654,27 +3694,23 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE_QUANTITY_INVALID</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>INVALID_QUANTITY, QUANTITY_INVALID</t>
-        </is>
-      </c>
+          <t>EDIFACT_LINE_INTEGRITY_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr"/>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Article Quantity Invalid</t>
+          <t>Edifact Line Integrity Mismatch</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Une ou plusieurs quantités article sont invalides.</t>
+          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3684,12 +3720,12 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -3699,7 +3735,7 @@
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
@@ -3729,17 +3765,17 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>Une ou plusieurs quantités article sont invalides.</t>
+          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
         </is>
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>One or more article quantities are invalid.</t>
+          <t>The EDIFACT line integrity check failed.</t>
         </is>
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S31" s="4" t="inlineStr"/>
@@ -3758,32 +3794,28 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W31" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : INVALID_QUANTITY, QUANTITY_INVALID</t>
-        </is>
-      </c>
+      <c r="W31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>UNIT_PRICE_MISSING</t>
+          <t>EDIFACT_NAD_DP_MISMATCH</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr"/>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Unit Price Missing</t>
+          <t>Edifact Nad Dp Mismatch</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs prix unitaires sont manquants.</t>
+          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -3793,12 +3825,12 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -3808,7 +3840,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -3838,17 +3870,17 @@
       </c>
       <c r="P32" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs prix unitaires sont manquants.</t>
+          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
         </is>
       </c>
       <c r="Q32" s="4" t="inlineStr">
         <is>
-          <t>One or more unit prices are missing.</t>
+          <t>The selected SHIP-TO does not match the generated NAD+DP segment.</t>
         </is>
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S32" s="4" t="inlineStr"/>
@@ -3872,33 +3904,33 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_LINE_INTEGRITY_MISMATCH</t>
+          <t>DUPLICATE_ALREADY_SENT</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Edifact Line Integrity Mismatch</t>
+          <t>Duplicate Already Sent</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
+          <t>Cette commande a déjà été traitée et envoyée.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>EDI_VALIDATION</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Métier / idempotence</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -3913,7 +3945,7 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
@@ -3923,12 +3955,12 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
@@ -3943,17 +3975,17 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
+          <t>Cette commande a déjà été traitée et envoyée.</t>
         </is>
       </c>
       <c r="Q33" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT line integrity check failed.</t>
+          <t>This order has already been processed and sent.</t>
         </is>
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
+          <t>src/file2edi/store.py</t>
         </is>
       </c>
       <c r="S33" s="4" t="inlineStr"/>
@@ -3977,33 +4009,37 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_NAD_DP_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr"/>
+          <t>NO_DELIVERY_ADDRESS</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>CONTRACT_BREAK_ADDRESSES_MISSING</t>
+        </is>
+      </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Edifact Nad Dp Mismatch</t>
+          <t>No Delivery Address</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
+          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>EDI_VALIDATION</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Référentiel / matching</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -4018,7 +4054,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -4048,20 +4084,24 @@
       </c>
       <c r="P34" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
+          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
         </is>
       </c>
       <c r="Q34" s="4" t="inlineStr">
         <is>
-          <t>The selected SHIP-TO does not match the generated NAD+DP segment.</t>
+          <t>No delivery address was detected in the document.</t>
         </is>
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
-        </is>
-      </c>
-      <c r="S34" s="4" t="inlineStr"/>
+          <t>app/engines/rejection_engine.py</t>
+        </is>
+      </c>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>_check_delivery_address</t>
+        </is>
+      </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4074,41 +4114,45 @@
       </c>
       <c r="V34" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W34" s="4" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="W34" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CONTRACT_BREAK_ADDRESSES_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE_ALREADY_SENT</t>
+          <t>ARTICLE_NOT_FOUND</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Duplicate Already Sent</t>
+          <t>Article Not Found</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Cette commande a déjà été traitée et envoyée.</t>
+          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY</t>
+          <t>BUSINESS_VALIDATION</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Métier / idempotence</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -4133,12 +4177,12 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
@@ -4153,20 +4197,24 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>Cette commande a déjà été traitée et envoyée.</t>
+          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
         </is>
       </c>
       <c r="Q35" s="4" t="inlineStr">
         <is>
-          <t>This order has already been processed and sent.</t>
+          <t>One or more article codes were not found in the materials master.</t>
         </is>
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
-          <t>src/file2edi/store.py</t>
-        </is>
-      </c>
-      <c r="S35" s="4" t="inlineStr"/>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
+        </is>
+      </c>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>_check_line_items</t>
+        </is>
+      </c>
       <c r="T35" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4179,7 +4227,7 @@
       </c>
       <c r="V35" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="W35" s="4" t="inlineStr"/>
@@ -4187,33 +4235,33 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY_ADDRESS_INVALID</t>
+          <t>PO_NUMBER_DUPLICATE</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Delivery Address Invalid</t>
+          <t>Po Number Duplicate</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>L'adresse de livraison n'a pas pu être associée aux données maîtres en raison d'une mauvaise détection ou de données client manquantes.</t>
+          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>BUSINESS_VALIDATION</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Métier / idempotence</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -4223,12 +4271,12 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
@@ -4238,17 +4286,17 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Mettre en revue</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
@@ -4258,22 +4306,22 @@
       </c>
       <c r="P36" s="4" t="inlineStr">
         <is>
-          <t>L'adresse de livraison n'a pas pu être associée aux données maîtres en raison d'une mauvaise détection ou de données client manquantes.</t>
+          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
         </is>
       </c>
       <c r="Q36" s="4" t="inlineStr">
         <is>
-          <t>The delivery address could not be matched to master data due to poor detection or missing customer data.</t>
+          <t>This purchase order number already exists in the SAP sales order history.</t>
         </is>
       </c>
       <c r="R36" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>src/file2edi/store.py</t>
         </is>
       </c>
       <c r="S36" s="4" t="inlineStr">
         <is>
-          <t>_check_delivery_address</t>
+          <t>_check_po_duplicate</t>
         </is>
       </c>
       <c r="T36" s="4" t="inlineStr">
@@ -4296,33 +4344,33 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>NO_DELIVERY_ADDRESS</t>
+          <t>NOT_AN_ORDER</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>No Delivery Address</t>
+          <t>Not An Order</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
+          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>CLASSIFICATION</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Structurelle / classification</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -4347,7 +4395,7 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
@@ -4367,22 +4415,22 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
+          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
         </is>
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
-          <t>No delivery address was detected in the document.</t>
+          <t>The submitted document is not a purchase order (contract, quote, proforma…).</t>
         </is>
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/extraction.py</t>
         </is>
       </c>
       <c r="S37" s="4" t="inlineStr">
         <is>
-          <t>_check_delivery_address</t>
+          <t>_check_document_type</t>
         </is>
       </c>
       <c r="T37" s="4" t="inlineStr">
@@ -4405,18 +4453,22 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr"/>
+          <t>NO_LINE_ITEMS</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>NO_ORDER_LINES</t>
+        </is>
+      </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Article Not Found</t>
+          <t>No Line Items</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
+          <t>Aucune ligne article n'a été trouvée dans le document.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -4426,7 +4478,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>BUSINESS_VALIDATION</t>
+          <t>EXTRACTION</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -4476,12 +4528,12 @@
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
+          <t>Aucune ligne article n'a été trouvée dans le document.</t>
         </is>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>One or more article codes were not found in the materials master.</t>
+          <t>No order line items were found in the document.</t>
         </is>
       </c>
       <c r="R38" s="4" t="inlineStr">
@@ -4509,28 +4561,32 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="W38" s="4" t="inlineStr"/>
+      <c r="W38" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : NO_ORDER_LINES</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>PO_NUMBER_DUPLICATE</t>
+          <t>QUANTITY_MISSING</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Po Number Duplicate</t>
+          <t>Quantity Missing</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
+          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -4540,22 +4596,22 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Métier / idempotence</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -4565,17 +4621,17 @@
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>Mettre en revue</t>
+          <t>Bloquer le traitement</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -4585,22 +4641,22 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
+          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="Q39" s="4" t="inlineStr">
         <is>
-          <t>This purchase order number already exists in the SAP sales order history.</t>
+          <t>Quantity is missing on one or more order lines.</t>
         </is>
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>src/file2edi/store.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S39" s="4" t="inlineStr">
         <is>
-          <t>_check_po_duplicate</t>
+          <t>_check_line_items</t>
         </is>
       </c>
       <c r="T39" s="4" t="inlineStr">
@@ -4623,38 +4679,38 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>CUSTOMER_NOT_DEFINED</t>
+          <t>PRICE_MISSING</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Customer Not Defined</t>
+          <t>Price Missing</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Aucun client (SOLD-TO) n'a pu être identifié dans les données maîtres.</t>
+          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -4674,12 +4730,12 @@
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
@@ -4694,22 +4750,22 @@
       </c>
       <c r="P40" s="4" t="inlineStr">
         <is>
-          <t>Aucun client (SOLD-TO) n'a pu être identifié dans les données maîtres.</t>
+          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="Q40" s="4" t="inlineStr">
         <is>
-          <t>No customer (SOLD-TO) could be identified in masterdata.</t>
+          <t>Unit price is missing on one or more order lines.</t>
         </is>
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S40" s="4" t="inlineStr">
         <is>
-          <t>_check_customer</t>
+          <t>_check_line_items</t>
         </is>
       </c>
       <c r="T40" s="4" t="inlineStr">
@@ -4732,33 +4788,33 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>NOT_AN_ORDER</t>
+          <t>DELIVERY_SFTP_FAILED</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Not An Order</t>
+          <t>Delivery Sftp Failed</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
+          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>DOCUMENT</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>CLASSIFICATION</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / classification</t>
+          <t>Intégration</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -4783,17 +4839,17 @@
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>DELIVERY_FAILED</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Relancer automatiquement puis escalader</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
@@ -4803,24 +4859,20 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
+          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
         </is>
       </c>
       <c r="Q41" s="4" t="inlineStr">
         <is>
-          <t>The submitted document is not a purchase order (contract, quote, proforma…).</t>
+          <t>The .tst file was generated but the SFTP delivery failed.</t>
         </is>
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>app/extraction.py</t>
-        </is>
-      </c>
-      <c r="S41" s="4" t="inlineStr">
-        <is>
-          <t>_check_document_type</t>
-        </is>
-      </c>
+          <t>src/sftp_delivery.py</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4833,7 +4885,7 @@
       </c>
       <c r="V41" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="W41" s="4" t="inlineStr"/>
@@ -4841,37 +4893,33 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>NO_LINE_ITEMS</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>NO_ORDER_LINES</t>
-        </is>
-      </c>
+          <t>DELIVERY_EMAIL_FAILED</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr"/>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>No Line Items</t>
+          <t>Delivery Email Failed</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article n'a été trouvée dans le document.</t>
+          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>EXTRACTION</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Intégration</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -4901,12 +4949,12 @@
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>DELIVERY_FAILED</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Relancer automatiquement puis escalader</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
@@ -4916,24 +4964,20 @@
       </c>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article n'a été trouvée dans le document.</t>
+          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
         </is>
       </c>
       <c r="Q42" s="4" t="inlineStr">
         <is>
-          <t>No order line items were found in the document.</t>
+          <t>The .tst file was generated but the email delivery failed.</t>
         </is>
       </c>
       <c r="R42" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S42" s="4" t="inlineStr">
-        <is>
-          <t>_check_line_items</t>
-        </is>
-      </c>
+          <t>src/sftp_delivery.py</t>
+        </is>
+      </c>
+      <c r="S42" s="4" t="inlineStr"/>
       <c r="T42" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4946,60 +4990,56 @@
       </c>
       <c r="V42" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="W42" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : NO_ORDER_LINES</t>
-        </is>
-      </c>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="W42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>QUANTITY_MISSING</t>
+          <t>SOLDTO_CONFIDENCE_MIN</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Quantity Missing</t>
+          <t>Seuil de confiance Sold-to</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
+          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>BUSINESS_VALIDATION</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Matching</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
@@ -5019,96 +5059,88 @@
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Mettre en revue si implémenté</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
+          <t>Confirmer le client</t>
         </is>
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
+          <t>Confiance Sold-to insuffisante</t>
         </is>
       </c>
       <c r="Q43" s="4" t="inlineStr">
         <is>
-          <t>Quantity is missing on one or more order lines.</t>
+          <t>Sold-to confidence below threshold</t>
         </is>
       </c>
       <c r="R43" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S43" s="4" t="inlineStr">
-        <is>
-          <t>_check_line_items</t>
-        </is>
-      </c>
-      <c r="T43" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U43" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+          <t>Documentation uniquement</t>
+        </is>
+      </c>
+      <c r="S43" s="4" t="inlineStr"/>
+      <c r="T43" s="4" t="inlineStr"/>
+      <c r="U43" s="4" t="inlineStr"/>
       <c r="V43" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="W43" s="4" t="inlineStr"/>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="W43" s="4" t="inlineStr">
+        <is>
+          <t>Critère documenté, pas un code du catalogue.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>PRICE_MISSING</t>
+          <t>SHIPTO_CONFIDENCE_MIN</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr"/>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Price Missing</t>
+          <t>Seuil de confiance Ship-to</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
+          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Matching</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
@@ -5128,469 +5160,49 @@
       </c>
       <c r="N44" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Mettre en revue si implémenté</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
+          <t>Confirmer l'adresse</t>
         </is>
       </c>
       <c r="P44" s="4" t="inlineStr">
         <is>
-          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
+          <t>Confiance Ship-to insuffisante</t>
         </is>
       </c>
       <c r="Q44" s="4" t="inlineStr">
         <is>
-          <t>Unit price is missing on one or more order lines.</t>
+          <t>Ship-to confidence below threshold</t>
         </is>
       </c>
       <c r="R44" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S44" s="4" t="inlineStr">
-        <is>
-          <t>_check_line_items</t>
-        </is>
-      </c>
-      <c r="T44" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U44" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+          <t>Documentation uniquement</t>
+        </is>
+      </c>
+      <c r="S44" s="4" t="inlineStr"/>
+      <c r="T44" s="4" t="inlineStr"/>
+      <c r="U44" s="4" t="inlineStr"/>
       <c r="V44" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="W44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY_SFTP_FAILED</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Delivery Sftp Failed</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Intégration</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>ORDER</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY_FAILED</t>
-        </is>
-      </c>
-      <c r="N45" s="4" t="inlineStr">
-        <is>
-          <t>Relancer automatiquement puis escalader</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="inlineStr">
-        <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
-        </is>
-      </c>
-      <c r="P45" s="4" t="inlineStr">
-        <is>
-          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
-        </is>
-      </c>
-      <c r="Q45" s="4" t="inlineStr">
-        <is>
-          <t>The .tst file was generated but the SFTP delivery failed.</t>
-        </is>
-      </c>
-      <c r="R45" s="4" t="inlineStr">
-        <is>
-          <t>src/sftp_delivery.py</t>
-        </is>
-      </c>
-      <c r="S45" s="4" t="inlineStr"/>
-      <c r="T45" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U45" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="V45" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY_EMAIL_FAILED</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr"/>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Delivery Email Failed</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>Intégration</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>ORDER</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L46" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M46" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY_FAILED</t>
-        </is>
-      </c>
-      <c r="N46" s="4" t="inlineStr">
-        <is>
-          <t>Relancer automatiquement puis escalader</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
-        </is>
-      </c>
-      <c r="P46" s="4" t="inlineStr">
-        <is>
-          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
-        </is>
-      </c>
-      <c r="Q46" s="4" t="inlineStr">
-        <is>
-          <t>The .tst file was generated but the email delivery failed.</t>
-        </is>
-      </c>
-      <c r="R46" s="4" t="inlineStr">
-        <is>
-          <t>src/sftp_delivery.py</t>
-        </is>
-      </c>
-      <c r="S46" s="4" t="inlineStr"/>
-      <c r="T46" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U46" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="V46" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>SOLDTO_CONFIDENCE_MIN</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Seuil de confiance Sold-to</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>PARTNER</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>MATCHING</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>ORDER</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L47" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M47" s="4" t="inlineStr">
-        <is>
-          <t>PENDING_USER_INPUT</t>
-        </is>
-      </c>
-      <c r="N47" s="4" t="inlineStr">
-        <is>
-          <t>Mettre en revue si implémenté</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>Confirmer le client</t>
-        </is>
-      </c>
-      <c r="P47" s="4" t="inlineStr">
-        <is>
-          <t>Confiance Sold-to insuffisante</t>
-        </is>
-      </c>
-      <c r="Q47" s="4" t="inlineStr">
-        <is>
-          <t>Sold-to confidence below threshold</t>
-        </is>
-      </c>
-      <c r="R47" s="4" t="inlineStr">
-        <is>
-          <t>Documentation uniquement</t>
-        </is>
-      </c>
-      <c r="S47" s="4" t="inlineStr"/>
-      <c r="T47" s="4" t="inlineStr"/>
-      <c r="U47" s="4" t="inlineStr"/>
-      <c r="V47" s="4" t="inlineStr">
-        <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="W47" s="4" t="inlineStr">
+      <c r="W44" s="4" t="inlineStr">
         <is>
           <t>Critère documenté, pas un code du catalogue.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>SHIPTO_CONFIDENCE_MIN</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Seuil de confiance Ship-to</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>PARTNER</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>MATCHING</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M48" s="4" t="inlineStr">
-        <is>
-          <t>PENDING_USER_INPUT</t>
-        </is>
-      </c>
-      <c r="N48" s="4" t="inlineStr">
-        <is>
-          <t>Mettre en revue si implémenté</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>Confirmer l'adresse</t>
-        </is>
-      </c>
-      <c r="P48" s="4" t="inlineStr">
-        <is>
-          <t>Confiance Ship-to insuffisante</t>
-        </is>
-      </c>
-      <c r="Q48" s="4" t="inlineStr">
-        <is>
-          <t>Ship-to confidence below threshold</t>
-        </is>
-      </c>
-      <c r="R48" s="4" t="inlineStr">
-        <is>
-          <t>Documentation uniquement</t>
-        </is>
-      </c>
-      <c r="S48" s="4" t="inlineStr"/>
-      <c r="T48" s="4" t="inlineStr"/>
-      <c r="U48" s="4" t="inlineStr"/>
-      <c r="V48" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="W48" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté, pas un code du catalogue.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:W48"/>
+  <autoFilter ref="A2:W44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:W1"/>
   </mergeCells>
-  <conditionalFormatting sqref="I3:I48">
+  <conditionalFormatting sqref="I3:I44">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Oui"</formula>
     </cfRule>
@@ -5642,7 +5254,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -5652,7 +5264,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -5672,7 +5284,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -5682,7 +5294,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -5778,7 +5390,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -5824,7 +5436,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -5844,7 +5456,7 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: optimize validation code classes
</commit_message>
<xml_diff>
--- a/docs/validation_rules_inventory.xlsx
+++ b/docs/validation_rules_inventory.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Incohérences" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Règles'!$A$2:$W$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Règles'!$A$2:$W$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Incohérences'!$A$2:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -172,8 +172,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationRules" displayName="ValidationRules" ref="A2:W44" headerRowCount="1">
-  <autoFilter ref="A2:W44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationRules" displayName="ValidationRules" ref="A2:W42" headerRowCount="1">
+  <autoFilter ref="A2:W42"/>
   <tableColumns count="23">
     <tableColumn id="1" name="Code canonique"/>
     <tableColumn id="2" name="Alias / anciens codes"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W44"/>
+  <dimension ref="A1:W42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2184,33 +2184,37 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>CONTRACT_BREAK_ARTICLES_MISSING</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr"/>
+          <t>SOLDTO_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
+        </is>
+      </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Contract Break Articles Missing</t>
+          <t>Soldto Not Found</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article exploitable n'a été trouvée.</t>
+          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>EXTRACTION</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Référentiel / matching</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -2255,20 +2259,24 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article exploitable n'a été trouvée.</t>
+          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>No usable order line item was found.</t>
+          <t>No matching SOLD-TO was found in master data.</t>
         </is>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S17" s="4" t="inlineStr"/>
+          <t>app/engines/rejection_engine.py</t>
+        </is>
+      </c>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>_check_customer</t>
+        </is>
+      </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2281,30 +2289,30 @@
       </c>
       <c r="V17" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W17" s="4" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>SOLDTO_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
-        </is>
-      </c>
+          <t>SOLDTO_AMBIGUOUS_MATCH</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Soldto Not Found</t>
+          <t>Soldto Ambiguous Match</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
+          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -2364,12 +2372,12 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Aucun SOLD-TO correspondant n'a été trouvé dans les données maîtres.</t>
+          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>No matching SOLD-TO was found in master data.</t>
+          <t>Multiple SOLD-TO candidates matched with equivalent confidence.</t>
         </is>
       </c>
       <c r="R18" s="4" t="inlineStr">
@@ -2377,11 +2385,7 @@
           <t>app/engines/rejection_engine.py</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>_check_customer</t>
-        </is>
-      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2394,30 +2398,30 @@
       </c>
       <c r="V18" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : CUSTOMER_NOT_DEFINED, CONTRACT_BREAK_SOLDTO_MISSING</t>
-        </is>
-      </c>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>SOLDTO_AMBIGUOUS_MATCH</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
+          <t>SHIPTO_CANDIDATES_MISSING</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
+        </is>
+      </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Soldto Ambiguous Match</t>
+          <t>Shipto Candidates Missing</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
+          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2457,12 +2461,12 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -2477,12 +2481,12 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SOLD-TO correspondent avec une confiance équivalente.</t>
+          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>Multiple SOLD-TO candidates matched with equivalent confidence.</t>
+          <t>No SHIP-TO candidate exists in the current SOLD-TO family.</t>
         </is>
       </c>
       <c r="R19" s="4" t="inlineStr">
@@ -2506,27 +2510,31 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_CANDIDATES_MISSING</t>
+          <t>SHIPTO_NO_STRONG_MATCH</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
+          <t>SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Shipto Candidates Missing</t>
+          <t>Shipto No Strong Match</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
+          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2566,12 +2574,12 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -2586,12 +2594,12 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>Aucun candidat SHIP-TO n'existe dans la famille du SOLD-TO courant.</t>
+          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>No SHIP-TO candidate exists in the current SOLD-TO family.</t>
+          <t>SHIP-TO candidates exist but none matched with strong evidence.</t>
         </is>
       </c>
       <c r="R20" s="4" t="inlineStr">
@@ -2599,7 +2607,11 @@
           <t>app/engines/rejection_engine.py</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>_check_delivery_address</t>
+        </is>
+      </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2612,34 +2624,30 @@
       </c>
       <c r="V20" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
         <is>
-          <t>Alias normalisés : CONTRACT_BREAK_SHIPTO_CANDIDATES_MISSING</t>
+          <t>Alias normalisés : SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_NO_STRONG_MATCH</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
-        </is>
-      </c>
+          <t>SHIPTO_AMBIGUOUS_MATCH</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr"/>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Shipto No Strong Match</t>
+          <t>Shipto Ambiguous Match</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
+          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2699,12 +2707,12 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>Des candidats SHIP-TO existent mais aucun ne correspond avec une preuve forte.</t>
+          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
         </is>
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>SHIP-TO candidates exist but none matched with strong evidence.</t>
+          <t>Multiple SHIP-TO candidates matched with equivalent strong evidence.</t>
         </is>
       </c>
       <c r="R21" s="4" t="inlineStr">
@@ -2712,11 +2720,7 @@
           <t>app/engines/rejection_engine.py</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>_check_delivery_address</t>
-        </is>
-      </c>
+      <c r="S21" s="4" t="inlineStr"/>
       <c r="T21" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -2729,30 +2733,26 @@
       </c>
       <c r="V21" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="W21" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : SHIPTO_MISSING, DELIVERY_ADDRESS_INVALID, SHIPTO_MASTERDATA_MISMATCH, SHIPTO_WEAK_EVIDENCE_IN_SOLDTO_FAMILY</t>
-        </is>
-      </c>
+          <t>À vérifier</t>
+        </is>
+      </c>
+      <c r="W21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_AMBIGUOUS_MATCH</t>
+          <t>SHIPTO_SOLDTO_MISMATCH</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Shipto Ambiguous Match</t>
+          <t>Shipto Soldto Mismatch</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
+          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2792,12 +2792,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -2812,12 +2812,12 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Plusieurs SHIP-TO correspondent avec une preuve forte équivalente.</t>
+          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>Multiple SHIP-TO candidates matched with equivalent strong evidence.</t>
+          <t>The selected SHIP-TO does not belong to the current SOLD-TO family.</t>
         </is>
       </c>
       <c r="R22" s="4" t="inlineStr">
@@ -2846,33 +2846,33 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>SHIPTO_SOLDTO_MISMATCH</t>
+          <t>EDIFACT_MISSING_BGM</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr"/>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Shipto Soldto Mismatch</t>
+          <t>Edifact Missing Bgm</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
+          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>EDI_VALIDATION</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -2917,17 +2917,17 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné n'appartient pas à la famille du SOLD-TO courant.</t>
+          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
         </is>
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>The selected SHIP-TO does not belong to the current SOLD-TO family.</t>
+          <t>The EDIFACT BGM segment is missing the mandatory order reference.</t>
         </is>
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S23" s="4" t="inlineStr"/>
@@ -2951,18 +2951,18 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_BGM</t>
+          <t>EDIFACT_MISSING_DTM_137</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr"/>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Bgm</t>
+          <t>Edifact Missing Dtm 137</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
+          <t>La date document DTM+137 est manquante ou invalide.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>Le segment EDIFACT BGM ne contient pas la référence de commande obligatoire.</t>
+          <t>La date document DTM+137 est manquante ou invalide.</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT BGM segment is missing the mandatory order reference.</t>
+          <t>The DTM+137 document date is missing or invalid.</t>
         </is>
       </c>
       <c r="R24" s="4" t="inlineStr">
@@ -3056,18 +3056,18 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_DTM_137</t>
+          <t>EDIFACT_MISSING_NAD_BY</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Dtm 137</t>
+          <t>Edifact Missing Nad By</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>La date document DTM+137 est manquante ou invalide.</t>
+          <t>Le segment acheteur NAD+BY est incomplet.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -3127,12 +3127,12 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>La date document DTM+137 est manquante ou invalide.</t>
+          <t>Le segment acheteur NAD+BY est incomplet.</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>The DTM+137 document date is missing or invalid.</t>
+          <t>The buyer NAD+BY segment is incomplete.</t>
         </is>
       </c>
       <c r="R25" s="4" t="inlineStr">
@@ -3161,18 +3161,18 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_NAD_BY</t>
+          <t>EDIFACT_MISSING_NAD_DP</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr"/>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Nad By</t>
+          <t>Edifact Missing Nad Dp</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Le segment acheteur NAD+BY est incomplet.</t>
+          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -3232,12 +3232,12 @@
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>Le segment acheteur NAD+BY est incomplet.</t>
+          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
         </is>
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>The buyer NAD+BY segment is incomplete.</t>
+          <t>The delivery NAD+DP segment is incomplete or unresolved.</t>
         </is>
       </c>
       <c r="R26" s="4" t="inlineStr">
@@ -3266,18 +3266,18 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_NAD_DP</t>
+          <t>EDIFACT_MISSING_LIN</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Nad Dp</t>
+          <t>Edifact Missing Lin</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
+          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -3337,12 +3337,12 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>Le segment livraison NAD+DP est incomplet ou non résolu.</t>
+          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
         </is>
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>The delivery NAD+DP segment is incomplete or unresolved.</t>
+          <t>The EDIFACT line segments LIN/PIA/IMD/QTY/PRI are missing or incomplete.</t>
         </is>
       </c>
       <c r="R27" s="4" t="inlineStr">
@@ -3371,23 +3371,27 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_MISSING_LIN</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr"/>
+          <t>ARTICLE_QUANTITY_INVALID</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>INVALID_QUANTITY, QUANTITY_INVALID</t>
+        </is>
+      </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Edifact Missing Lin</t>
+          <t>Article Quantity Invalid</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
+          <t>Une ou plusieurs quantités article sont invalides.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -3397,12 +3401,12 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -3412,7 +3416,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
@@ -3442,17 +3446,17 @@
       </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
-          <t>Les segments lignes EDIFACT LIN/PIA/IMD/QTY/PRI sont manquants ou incomplets.</t>
+          <t>Une ou plusieurs quantités article sont invalides.</t>
         </is>
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT line segments LIN/PIA/IMD/QTY/PRI are missing or incomplete.</t>
+          <t>One or more article quantities are invalid.</t>
         </is>
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S28" s="4" t="inlineStr"/>
@@ -3471,27 +3475,31 @@
           <t>À vérifier</t>
         </is>
       </c>
-      <c r="W28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : INVALID_QUANTITY, QUANTITY_INVALID</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE_QUANTITY_INVALID</t>
+          <t>UNIT_PRICE_MISSING</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>INVALID_QUANTITY, QUANTITY_INVALID</t>
+          <t>PRICE_MISSING</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Article Quantity Invalid</t>
+          <t>Unit Price Missing</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Une ou plusieurs quantités article sont invalides.</t>
+          <t>Un ou plusieurs prix unitaires sont manquants.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -3551,12 +3559,12 @@
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>Une ou plusieurs quantités article sont invalides.</t>
+          <t>Un ou plusieurs prix unitaires sont manquants.</t>
         </is>
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>One or more article quantities are invalid.</t>
+          <t>One or more unit prices are missing.</t>
         </is>
       </c>
       <c r="R29" s="4" t="inlineStr">
@@ -3564,7 +3572,11 @@
           <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr">
+        <is>
+          <t>_check_line_items</t>
+        </is>
+      </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -3577,35 +3589,35 @@
       </c>
       <c r="V29" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="W29" s="4" t="inlineStr">
         <is>
-          <t>Alias normalisés : INVALID_QUANTITY, QUANTITY_INVALID</t>
+          <t>Alias normalisés : PRICE_MISSING</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>UNIT_PRICE_MISSING</t>
+          <t>EDIFACT_LINE_INTEGRITY_MISMATCH</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr"/>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Unit Price Missing</t>
+          <t>Edifact Line Integrity Mismatch</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs prix unitaires sont manquants.</t>
+          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>EDI</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3615,12 +3627,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Structurelle / cohérence EDI</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -3630,7 +3642,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
@@ -3660,17 +3672,17 @@
       </c>
       <c r="P30" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs prix unitaires sont manquants.</t>
+          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
         </is>
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>One or more unit prices are missing.</t>
+          <t>The EDIFACT line integrity check failed.</t>
         </is>
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
+          <t>app/edifact_generator.py</t>
         </is>
       </c>
       <c r="S30" s="4" t="inlineStr"/>
@@ -3694,18 +3706,18 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_LINE_INTEGRITY_MISMATCH</t>
+          <t>EDIFACT_NAD_DP_MISMATCH</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr"/>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Edifact Line Integrity Mismatch</t>
+          <t>Edifact Nad Dp Mismatch</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
+          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -3765,12 +3777,12 @@
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
-          <t>La cohérence des lignes EDIFACT est incorrecte.</t>
+          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
         </is>
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>The EDIFACT line integrity check failed.</t>
+          <t>The selected SHIP-TO does not match the generated NAD+DP segment.</t>
         </is>
       </c>
       <c r="R31" s="4" t="inlineStr">
@@ -3799,33 +3811,33 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>EDIFACT_NAD_DP_MISMATCH</t>
+          <t>DUPLICATE_ALREADY_SENT</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr"/>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Edifact Nad Dp Mismatch</t>
+          <t>Duplicate Already Sent</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
+          <t>Cette commande a déjà été traitée et envoyée.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>EDI</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>EDI_VALIDATION</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / cohérence EDI</t>
+          <t>Métier / idempotence</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -3840,7 +3852,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -3850,12 +3862,12 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -3870,17 +3882,17 @@
       </c>
       <c r="P32" s="4" t="inlineStr">
         <is>
-          <t>Le SHIP-TO sélectionné ne correspond pas au segment NAD+DP généré.</t>
+          <t>Cette commande a déjà été traitée et envoyée.</t>
         </is>
       </c>
       <c r="Q32" s="4" t="inlineStr">
         <is>
-          <t>The selected SHIP-TO does not match the generated NAD+DP segment.</t>
+          <t>This order has already been processed and sent.</t>
         </is>
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>app/edifact_generator.py</t>
+          <t>src/file2edi/store.py</t>
         </is>
       </c>
       <c r="S32" s="4" t="inlineStr"/>
@@ -3904,33 +3916,37 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE_ALREADY_SENT</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr"/>
+          <t>NO_DELIVERY_ADDRESS</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>CONTRACT_BREAK_ADDRESSES_MISSING</t>
+        </is>
+      </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Duplicate Already Sent</t>
+          <t>No Delivery Address</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Cette commande a déjà été traitée et envoyée.</t>
+          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Métier / idempotence</t>
+          <t>Référentiel / matching</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -3955,12 +3971,12 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
@@ -3975,20 +3991,24 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>Cette commande a déjà été traitée et envoyée.</t>
+          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
         </is>
       </c>
       <c r="Q33" s="4" t="inlineStr">
         <is>
-          <t>This order has already been processed and sent.</t>
+          <t>No delivery address was detected in the document.</t>
         </is>
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>src/file2edi/store.py</t>
-        </is>
-      </c>
-      <c r="S33" s="4" t="inlineStr"/>
+          <t>app/engines/rejection_engine.py</t>
+        </is>
+      </c>
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>_check_delivery_address</t>
+        </is>
+      </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4001,45 +4021,45 @@
       </c>
       <c r="V33" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W33" s="4" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="W33" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : CONTRACT_BREAK_ADDRESSES_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>NO_DELIVERY_ADDRESS</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>CONTRACT_BREAK_ADDRESSES_MISSING</t>
-        </is>
-      </c>
+          <t>ARTICLE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>No Delivery Address</t>
+          <t>Article Not Found</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
+          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>PARTNER</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>MATCHING</t>
+          <t>BUSINESS_VALIDATION</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / matching</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -4069,7 +4089,7 @@
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
@@ -4084,22 +4104,22 @@
       </c>
       <c r="P34" s="4" t="inlineStr">
         <is>
-          <t>Aucune adresse de livraison n'a été détectée dans le document.</t>
+          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
         </is>
       </c>
       <c r="Q34" s="4" t="inlineStr">
         <is>
-          <t>No delivery address was detected in the document.</t>
+          <t>One or more article codes were not found in the materials master.</t>
         </is>
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S34" s="4" t="inlineStr">
         <is>
-          <t>_check_delivery_address</t>
+          <t>_check_line_items</t>
         </is>
       </c>
       <c r="T34" s="4" t="inlineStr">
@@ -4117,32 +4137,28 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="W34" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : CONTRACT_BREAK_ADDRESSES_MISSING</t>
-        </is>
-      </c>
+      <c r="W34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE_NOT_FOUND</t>
+          <t>PO_NUMBER_DUPLICATE</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Article Not Found</t>
+          <t>Po Number Duplicate</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
+          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -4152,7 +4168,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Métier / idempotence</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -4162,12 +4178,12 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
@@ -4177,17 +4193,17 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>DUPLICATE</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Mettre en revue</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
@@ -4197,22 +4213,22 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>Un ou plusieurs codes articles sont introuvables dans le référentiel matières.</t>
+          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
         </is>
       </c>
       <c r="Q35" s="4" t="inlineStr">
         <is>
-          <t>One or more article codes were not found in the materials master.</t>
+          <t>This purchase order number already exists in the SAP sales order history.</t>
         </is>
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
+          <t>src/file2edi/store.py</t>
         </is>
       </c>
       <c r="S35" s="4" t="inlineStr">
         <is>
-          <t>_check_line_items</t>
+          <t>_check_po_duplicate</t>
         </is>
       </c>
       <c r="T35" s="4" t="inlineStr">
@@ -4235,33 +4251,33 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>PO_NUMBER_DUPLICATE</t>
+          <t>NOT_AN_ORDER</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Po Number Duplicate</t>
+          <t>Not An Order</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
+          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>BUSINESS_VALIDATION</t>
+          <t>CLASSIFICATION</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Métier / idempotence</t>
+          <t>Structurelle / classification</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -4271,32 +4287,32 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>DUPLICATE</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Mettre en revue</t>
+          <t>Bloquer le traitement</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
@@ -4306,22 +4322,22 @@
       </c>
       <c r="P36" s="4" t="inlineStr">
         <is>
-          <t>Ce numéro de commande existe déjà dans l'historique SAP.</t>
+          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
         </is>
       </c>
       <c r="Q36" s="4" t="inlineStr">
         <is>
-          <t>This purchase order number already exists in the SAP sales order history.</t>
+          <t>The submitted document is not a purchase order (contract, quote, proforma…).</t>
         </is>
       </c>
       <c r="R36" s="4" t="inlineStr">
         <is>
-          <t>src/file2edi/store.py</t>
+          <t>app/extraction.py</t>
         </is>
       </c>
       <c r="S36" s="4" t="inlineStr">
         <is>
-          <t>_check_po_duplicate</t>
+          <t>_check_document_type</t>
         </is>
       </c>
       <c r="T36" s="4" t="inlineStr">
@@ -4344,33 +4360,37 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>NOT_AN_ORDER</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
+          <t>NO_LINE_ITEMS</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>NO_ORDER_LINES, CONTRACT_BREAK_ARTICLES_MISSING</t>
+        </is>
+      </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Not An Order</t>
+          <t>No Line Items</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
+          <t>Aucune ligne article n'a été trouvée dans le document.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>DOCUMENT</t>
+          <t>ARTICLE</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>CLASSIFICATION</t>
+          <t>EXTRACTION</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Structurelle / classification</t>
+          <t>Référentiel / métier</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -4395,12 +4415,12 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>REJECTED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -4415,22 +4435,22 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>Le document soumis n'est pas un bon de commande (contrat, devis, proforma…).</t>
+          <t>Aucune ligne article n'a été trouvée dans le document.</t>
         </is>
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
-          <t>The submitted document is not a purchase order (contract, quote, proforma…).</t>
+          <t>No order line items were found in the document.</t>
         </is>
       </c>
       <c r="R37" s="4" t="inlineStr">
         <is>
-          <t>app/extraction.py</t>
+          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
         </is>
       </c>
       <c r="S37" s="4" t="inlineStr">
         <is>
-          <t>_check_document_type</t>
+          <t>_check_line_items</t>
         </is>
       </c>
       <c r="T37" s="4" t="inlineStr">
@@ -4448,27 +4468,27 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="W37" s="4" t="inlineStr"/>
+      <c r="W37" s="4" t="inlineStr">
+        <is>
+          <t>Alias normalisés : NO_ORDER_LINES, CONTRACT_BREAK_ARTICLES_MISSING</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>NO_LINE_ITEMS</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>NO_ORDER_LINES</t>
-        </is>
-      </c>
+          <t>QUANTITY_MISSING</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>No Line Items</t>
+          <t>Quantity Missing</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article n'a été trouvée dans le document.</t>
+          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -4478,7 +4498,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>EXTRACTION</t>
+          <t>BUSINESS_VALIDATION</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -4488,7 +4508,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>ORDER</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -4528,12 +4548,12 @@
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>Aucune ligne article n'a été trouvée dans le document.</t>
+          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
         </is>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>No order line items were found in the document.</t>
+          <t>Quantity is missing on one or more order lines.</t>
         </is>
       </c>
       <c r="R38" s="4" t="inlineStr">
@@ -4561,47 +4581,43 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="W38" s="4" t="inlineStr">
-        <is>
-          <t>Alias normalisés : NO_ORDER_LINES</t>
-        </is>
-      </c>
+      <c r="W38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>QUANTITY_MISSING</t>
+          <t>DELIVERY_SFTP_FAILED</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Quantity Missing</t>
+          <t>Delivery Sftp Failed</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
+          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>BUSINESS_VALIDATION</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Intégration</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -4626,12 +4642,12 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>DELIVERY_FAILED</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Relancer automatiquement puis escalader</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
@@ -4641,24 +4657,20 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>La quantité est manquante sur une ou plusieurs lignes article.</t>
+          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
         </is>
       </c>
       <c r="Q39" s="4" t="inlineStr">
         <is>
-          <t>Quantity is missing on one or more order lines.</t>
+          <t>The .tst file was generated but the SFTP delivery failed.</t>
         </is>
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S39" s="4" t="inlineStr">
-        <is>
-          <t>_check_line_items</t>
-        </is>
-      </c>
+          <t>src/sftp_delivery.py</t>
+        </is>
+      </c>
+      <c r="S39" s="4" t="inlineStr"/>
       <c r="T39" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4671,7 +4683,7 @@
       </c>
       <c r="V39" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="W39" s="4" t="inlineStr"/>
@@ -4679,38 +4691,38 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>PRICE_MISSING</t>
+          <t>DELIVERY_EMAIL_FAILED</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Price Missing</t>
+          <t>Delivery Email Failed</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
+          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>ARTICLE</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>DELIVERY</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Référentiel / métier</t>
+          <t>Intégration</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>LINE</t>
+          <t>ORDER</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -4735,12 +4747,12 @@
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>PENDING_USER_INPUT</t>
+          <t>DELIVERY_FAILED</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>Bloquer le traitement</t>
+          <t>Relancer automatiquement puis escalader</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
@@ -4750,24 +4762,20 @@
       </c>
       <c r="P40" s="4" t="inlineStr">
         <is>
-          <t>Le prix unitaire est manquant sur une ou plusieurs lignes article.</t>
+          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
         </is>
       </c>
       <c r="Q40" s="4" t="inlineStr">
         <is>
-          <t>Unit price is missing on one or more order lines.</t>
+          <t>The .tst file was generated but the email delivery failed.</t>
         </is>
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>app/engines/rejection_engine.py; src/pompac_rules.py</t>
-        </is>
-      </c>
-      <c r="S40" s="4" t="inlineStr">
-        <is>
-          <t>_check_line_items</t>
-        </is>
-      </c>
+          <t>src/sftp_delivery.py</t>
+        </is>
+      </c>
+      <c r="S40" s="4" t="inlineStr"/>
       <c r="T40" s="4" t="inlineStr">
         <is>
           <t>tests/test_rejection_catalog.py</t>
@@ -4780,7 +4788,7 @@
       </c>
       <c r="V40" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="W40" s="4" t="inlineStr"/>
@@ -4788,33 +4796,33 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY_SFTP_FAILED</t>
+          <t>SOLDTO_CONFIDENCE_MIN</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Delivery Sftp Failed</t>
+          <t>Seuil de confiance Sold-to</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
+          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY</t>
+          <t>PARTNER</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY</t>
+          <t>MATCHING</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Intégration</t>
+          <t>Matching</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -4824,12 +4832,12 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
@@ -4844,97 +4852,93 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY_FAILED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
-          <t>Relancer automatiquement puis escalader</t>
+          <t>Mettre en revue si implémenté</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
+          <t>Confirmer le client</t>
         </is>
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>Le fichier .tst a été généré mais l'envoi SFTP a échoué.</t>
+          <t>Confiance Sold-to insuffisante</t>
         </is>
       </c>
       <c r="Q41" s="4" t="inlineStr">
         <is>
-          <t>The .tst file was generated but the SFTP delivery failed.</t>
+          <t>Sold-to confidence below threshold</t>
         </is>
       </c>
       <c r="R41" s="4" t="inlineStr">
         <is>
-          <t>src/sftp_delivery.py</t>
+          <t>Documentation uniquement</t>
         </is>
       </c>
       <c r="S41" s="4" t="inlineStr"/>
-      <c r="T41" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U41" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="T41" s="4" t="inlineStr"/>
+      <c r="U41" s="4" t="inlineStr"/>
       <c r="V41" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W41" s="4" t="inlineStr"/>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="W41" s="4" t="inlineStr">
+        <is>
+          <t>Critère documenté, pas un code du catalogue.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY_EMAIL_FAILED</t>
+          <t>SHIPTO_CONFIDENCE_MIN</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr"/>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Delivery Email Failed</t>
+          <t>Seuil de confiance Ship-to</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
+          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
+          <t>PARTNER</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>MATCHING</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Matching</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
           <t>DELIVERY</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>Intégration</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>ORDER</t>
-        </is>
-      </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>À vérifier</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -4949,260 +4953,54 @@
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>DELIVERY_FAILED</t>
+          <t>PENDING_USER_INPUT</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Relancer automatiquement puis escalader</t>
+          <t>Mettre en revue si implémenté</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>Corriger les données, le document ou le référentiel selon le contexte</t>
+          <t>Confirmer l'adresse</t>
         </is>
       </c>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>Le fichier .tst a été généré mais l'envoi email a échoué.</t>
+          <t>Confiance Ship-to insuffisante</t>
         </is>
       </c>
       <c r="Q42" s="4" t="inlineStr">
         <is>
-          <t>The .tst file was generated but the email delivery failed.</t>
+          <t>Ship-to confidence below threshold</t>
         </is>
       </c>
       <c r="R42" s="4" t="inlineStr">
         <is>
-          <t>src/sftp_delivery.py</t>
+          <t>Documentation uniquement</t>
         </is>
       </c>
       <c r="S42" s="4" t="inlineStr"/>
-      <c r="T42" s="4" t="inlineStr">
-        <is>
-          <t>tests/test_rejection_catalog.py</t>
-        </is>
-      </c>
-      <c r="U42" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
+      <c r="T42" s="4" t="inlineStr"/>
+      <c r="U42" s="4" t="inlineStr"/>
       <c r="V42" s="4" t="inlineStr">
         <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="W42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>SOLDTO_CONFIDENCE_MIN</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Seuil de confiance Sold-to</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>PARTNER</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>MATCHING</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>ORDER</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L43" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M43" s="4" t="inlineStr">
-        <is>
-          <t>PENDING_USER_INPUT</t>
-        </is>
-      </c>
-      <c r="N43" s="4" t="inlineStr">
-        <is>
-          <t>Mettre en revue si implémenté</t>
-        </is>
-      </c>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
-          <t>Confirmer le client</t>
-        </is>
-      </c>
-      <c r="P43" s="4" t="inlineStr">
-        <is>
-          <t>Confiance Sold-to insuffisante</t>
-        </is>
-      </c>
-      <c r="Q43" s="4" t="inlineStr">
-        <is>
-          <t>Sold-to confidence below threshold</t>
-        </is>
-      </c>
-      <c r="R43" s="4" t="inlineStr">
-        <is>
-          <t>Documentation uniquement</t>
-        </is>
-      </c>
-      <c r="S43" s="4" t="inlineStr"/>
-      <c r="T43" s="4" t="inlineStr"/>
-      <c r="U43" s="4" t="inlineStr"/>
-      <c r="V43" s="4" t="inlineStr">
-        <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="W43" s="4" t="inlineStr">
+      <c r="W42" s="4" t="inlineStr">
         <is>
           <t>Critère documenté, pas un code du catalogue.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>SHIPTO_CONFIDENCE_MIN</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Seuil de confiance Ship-to</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté de matching ; aucun code applicatif canonique trouvé.</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>PARTNER</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>MATCHING</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>DELIVERY</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>À vérifier</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="L44" s="4" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M44" s="4" t="inlineStr">
-        <is>
-          <t>PENDING_USER_INPUT</t>
-        </is>
-      </c>
-      <c r="N44" s="4" t="inlineStr">
-        <is>
-          <t>Mettre en revue si implémenté</t>
-        </is>
-      </c>
-      <c r="O44" s="4" t="inlineStr">
-        <is>
-          <t>Confirmer l'adresse</t>
-        </is>
-      </c>
-      <c r="P44" s="4" t="inlineStr">
-        <is>
-          <t>Confiance Ship-to insuffisante</t>
-        </is>
-      </c>
-      <c r="Q44" s="4" t="inlineStr">
-        <is>
-          <t>Ship-to confidence below threshold</t>
-        </is>
-      </c>
-      <c r="R44" s="4" t="inlineStr">
-        <is>
-          <t>Documentation uniquement</t>
-        </is>
-      </c>
-      <c r="S44" s="4" t="inlineStr"/>
-      <c r="T44" s="4" t="inlineStr"/>
-      <c r="U44" s="4" t="inlineStr"/>
-      <c r="V44" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="W44" s="4" t="inlineStr">
-        <is>
-          <t>Critère documenté, pas un code du catalogue.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:W44"/>
+  <autoFilter ref="A2:W42"/>
   <mergeCells count="1">
     <mergeCell ref="A1:W1"/>
   </mergeCells>
-  <conditionalFormatting sqref="I3:I44">
+  <conditionalFormatting sqref="I3:I42">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Oui"</formula>
     </cfRule>
@@ -5254,7 +5052,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -5264,7 +5062,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -5284,7 +5082,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
@@ -5330,7 +5128,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -5436,7 +5234,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23">

</xml_diff>